<commit_message>
Fix BeFinder upload SDG error
</commit_message>
<xml_diff>
--- a/Data/Raw Data/BeFinder/25LLB0001.xlsx
+++ b/Data/Raw Data/BeFinder/25LLB0001.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaleb.gordon\Desktop\LIMS\Data\Raw Data\BeFinder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE60A156-B7DC-4F6C-9C60-3F07DD945DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7E30838-A59B-4DCD-A758-65479B0E497E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D007E083-7497-45CA-B319-C1BAACA90E94}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="17">
   <si>
     <t>SAMPLE-001</t>
   </si>
@@ -75,13 +75,25 @@
   </si>
   <si>
     <t>SAMPLE-013</t>
+  </si>
+  <si>
+    <t>SAMPLE-014</t>
+  </si>
+  <si>
+    <t>SAMPLE-015</t>
+  </si>
+  <si>
+    <t>SAMPLE-016</t>
+  </si>
+  <si>
+    <t>SAMPLE-017</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -93,6 +105,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -117,10 +135,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32EB4217-35DD-4344-9522-5ADF1761370A}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="10.75" bestFit="1" customWidth="1"/>
@@ -588,14 +607,59 @@
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="2">
-        <v>677.01</v>
+      <c r="B12" s="3">
+        <v>879.51</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>1</v>
       </c>
     </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="3">
+        <v>520.89</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="3">
+        <v>798.74</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="3">
+        <v>542.16</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="3">
+        <v>624.73</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>